<commit_message>
Atualização nos experimentos 7 e 8
</commit_message>
<xml_diff>
--- a/Project_VIT/Main/Results/Experimento 7 - ViT/logs/train_log.xlsx
+++ b/Project_VIT/Main/Results/Experimento 7 - ViT/logs/train_log.xlsx
@@ -5,22 +5,22 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\RESULTS\logs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\marci_wawp\Desktop\Arquivos\Mestrado\Projeto-Classificadores\Project_VIT\Main\Results\Experimento 7 - ViT\logs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DF750BD-0C95-4B81-A6A9-18202C84C925}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D99B025-F727-4130-BCCF-8C12FA69FB0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="999999"/>
+  <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="5">
   <si>
     <t>epoch</t>
   </si>
@@ -41,11 +41,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial Unicode MS"/>
     </font>
   </fonts>
   <fills count="3">
@@ -74,10 +79,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3300,7 +3308,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="pt-BR"/>
-                  <a:t>Epocas</a:t>
+                  <a:t>Épocas</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -3418,7 +3426,7 @@
                 </a:pPr>
                 <a:r>
                   <a:rPr lang="pt-BR"/>
-                  <a:t>Acurácia</a:t>
+                  <a:t>Acurácia (%)</a:t>
                 </a:r>
               </a:p>
             </c:rich>
@@ -8202,7 +8210,7 @@
       <xdr:col>6</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>31</xdr:row>
-      <xdr:rowOff>4762</xdr:rowOff>
+      <xdr:rowOff>127000</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>18</xdr:col>
@@ -8559,15 +8567,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E501"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:W501"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="2" max="3" width="19.5703125" customWidth="1"/>
     <col min="4" max="4" width="15" customWidth="1"/>
     <col min="5" max="5" width="17.7109375" customWidth="1"/>
+    <col min="20" max="20" width="18.42578125" customWidth="1"/>
+    <col min="21" max="21" width="23.85546875" customWidth="1"/>
+    <col min="22" max="22" width="16.7109375" customWidth="1"/>
+    <col min="23" max="23" width="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" ht="30" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -8583,8 +8595,20 @@
       <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="U1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:23">
       <c r="A2">
         <v>0</v>
       </c>
@@ -8600,8 +8624,24 @@
       <c r="E2">
         <v>0.52708333353887005</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T2" s="2">
+        <f>AVERAGE(INDEX(B:B,(ROW(A1)-1)*100+2):INDEX(B:B,(ROW(A1)-1)*100+101))</f>
+        <v>0.45231027239595384</v>
+      </c>
+      <c r="U2">
+        <f>AVERAGE(INDEX(C:C,(ROW(A1)-1)*100+2):INDEX(C:C,(ROW(A1)-1)*100+101))</f>
+        <v>0.90469290345821307</v>
+      </c>
+      <c r="V2">
+        <f>AVERAGE(INDEX(D:D,(ROW(A1)-1)*100+2):INDEX(D:D,(ROW(A1)-1)*100+101))</f>
+        <v>0.65770371992569243</v>
+      </c>
+      <c r="W2">
+        <f>AVERAGE(INDEX(E:E,(ROW(A1)-1)*100+2):INDEX(E:E,(ROW(A1)-1)*100+101))</f>
+        <v>0.75984147557239401</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23">
       <c r="A3">
         <v>1</v>
       </c>
@@ -8617,8 +8657,24 @@
       <c r="E3">
         <v>0.66702586206896997</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T3" s="2">
+        <f>AVERAGE(INDEX(B:B,(ROW(A2)-1)*100+2):INDEX(B:B,(ROW(A2)-1)*100+101))</f>
+        <v>0.32653638017624176</v>
+      </c>
+      <c r="U3">
+        <f>AVERAGE(INDEX(C:C,(ROW(A2)-1)*100+2):INDEX(C:C,(ROW(A2)-1)*100+101))</f>
+        <v>0.98081141930835669</v>
+      </c>
+      <c r="V3">
+        <f>AVERAGE(INDEX(D:D,(ROW(A2)-1)*100+2):INDEX(D:D,(ROW(A2)-1)*100+101))</f>
+        <v>0.62962096961493497</v>
+      </c>
+      <c r="W3">
+        <f>AVERAGE(INDEX(E:E,(ROW(A2)-1)*100+2):INDEX(E:E,(ROW(A2)-1)*100+101))</f>
+        <v>0.79987284524687385</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23">
       <c r="A4">
         <v>2</v>
       </c>
@@ -8634,8 +8690,24 @@
       <c r="E4">
         <v>0.70193965544645998</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T4" s="2">
+        <f>AVERAGE(INDEX(B:B,(ROW(A3)-1)*100+2):INDEX(B:B,(ROW(A3)-1)*100+101))</f>
+        <v>0.30832203384435114</v>
+      </c>
+      <c r="U4">
+        <f>AVERAGE(INDEX(C:C,(ROW(A3)-1)*100+2):INDEX(C:C,(ROW(A3)-1)*100+101))</f>
+        <v>0.99090688040345765</v>
+      </c>
+      <c r="V4">
+        <f>AVERAGE(INDEX(D:D,(ROW(A3)-1)*100+2):INDEX(D:D,(ROW(A3)-1)*100+101))</f>
+        <v>0.60653110465612925</v>
+      </c>
+      <c r="W4">
+        <f>AVERAGE(INDEX(E:E,(ROW(A3)-1)*100+2):INDEX(E:E,(ROW(A3)-1)*100+101))</f>
+        <v>0.81417337233992881</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23">
       <c r="A5">
         <v>3</v>
       </c>
@@ -8651,8 +8723,24 @@
       <c r="E5">
         <v>0.67842433027837001</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T5" s="2">
+        <f>AVERAGE(INDEX(B:B,(ROW(A4)-1)*100+2):INDEX(B:B,(ROW(A4)-1)*100+101))</f>
+        <v>0.3015494109831901</v>
+      </c>
+      <c r="U5">
+        <f>AVERAGE(INDEX(C:C,(ROW(A4)-1)*100+2):INDEX(C:C,(ROW(A4)-1)*100+101))</f>
+        <v>0.99464967579250763</v>
+      </c>
+      <c r="V5">
+        <f>AVERAGE(INDEX(D:D,(ROW(A4)-1)*100+2):INDEX(D:D,(ROW(A4)-1)*100+101))</f>
+        <v>0.59083173984340542</v>
+      </c>
+      <c r="W5">
+        <f>AVERAGE(INDEX(E:E,(ROW(A4)-1)*100+2):INDEX(E:E,(ROW(A4)-1)*100+101))</f>
+        <v>0.82191594889794284</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23">
       <c r="A6">
         <v>4</v>
       </c>
@@ -8668,8 +8756,24 @@
       <c r="E6">
         <v>0.72071360171526</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T6" s="2">
+        <f>AVERAGE(INDEX(B:B,(ROW(A5)-1)*100+2):INDEX(B:B,(ROW(A5)-1)*100+101))</f>
+        <v>0.29766231004288263</v>
+      </c>
+      <c r="U6">
+        <f>AVERAGE(INDEX(C:C,(ROW(A5)-1)*100+2):INDEX(C:C,(ROW(A5)-1)*100+101))</f>
+        <v>0.99662824207492806</v>
+      </c>
+      <c r="V6">
+        <f>AVERAGE(INDEX(D:D,(ROW(A5)-1)*100+2):INDEX(D:D,(ROW(A5)-1)*100+101))</f>
+        <v>0.59167772869483104</v>
+      </c>
+      <c r="W6">
+        <f>AVERAGE(INDEX(E:E,(ROW(A5)-1)*100+2):INDEX(E:E,(ROW(A5)-1)*100+101))</f>
+        <v>0.82521216536390429</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23">
       <c r="A7">
         <v>5</v>
       </c>
@@ -8685,8 +8789,9 @@
       <c r="E7">
         <v>0.70234674352338999</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T7" s="2"/>
+    </row>
+    <row r="8" spans="1:23">
       <c r="A8">
         <v>6</v>
       </c>
@@ -8702,8 +8807,9 @@
       <c r="E8">
         <v>0.73283046004415997</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T8" s="2"/>
+    </row>
+    <row r="9" spans="1:23">
       <c r="A9">
         <v>7</v>
       </c>
@@ -8719,8 +8825,9 @@
       <c r="E9">
         <v>0.72492816119357995</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T9" s="2"/>
+    </row>
+    <row r="10" spans="1:23">
       <c r="A10">
         <v>8</v>
       </c>
@@ -8736,8 +8843,9 @@
       <c r="E10">
         <v>0.71420019179924998</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T10" s="2"/>
+    </row>
+    <row r="11" spans="1:23">
       <c r="A11">
         <v>9</v>
       </c>
@@ -8753,8 +8861,9 @@
       <c r="E11">
         <v>0.73544061320952003</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T11" s="2"/>
+    </row>
+    <row r="12" spans="1:23">
       <c r="A12">
         <v>10</v>
       </c>
@@ -8770,8 +8879,9 @@
       <c r="E12">
         <v>0.74729406148538002</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T12" s="2"/>
+    </row>
+    <row r="13" spans="1:23">
       <c r="A13">
         <v>11</v>
       </c>
@@ -8787,8 +8897,9 @@
       <c r="E13">
         <v>0.73682950214408005</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T13" s="2"/>
+    </row>
+    <row r="14" spans="1:23">
       <c r="A14">
         <v>12</v>
       </c>
@@ -8804,8 +8915,9 @@
       <c r="E14">
         <v>0.72497605386821995</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T14" s="2"/>
+    </row>
+    <row r="15" spans="1:23">
       <c r="A15">
         <v>13</v>
       </c>
@@ -8821,8 +8933,9 @@
       <c r="E15">
         <v>0.73678160946945004</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T15" s="2"/>
+    </row>
+    <row r="16" spans="1:23">
       <c r="A16">
         <v>14</v>
       </c>
@@ -8838,8 +8951,9 @@
       <c r="E16">
         <v>0.74724616881075001</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T16" s="2"/>
+    </row>
+    <row r="17" spans="1:20">
       <c r="A17">
         <v>15</v>
       </c>
@@ -8855,8 +8969,9 @@
       <c r="E17">
         <v>0.72749042168431</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T17" s="2"/>
+    </row>
+    <row r="18" spans="1:20">
       <c r="A18">
         <v>16</v>
       </c>
@@ -8872,8 +8987,9 @@
       <c r="E18">
         <v>0.75447796953136004</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T18" s="2"/>
+    </row>
+    <row r="19" spans="1:20">
       <c r="A19">
         <v>17</v>
       </c>
@@ -8889,8 +9005,9 @@
       <c r="E19">
         <v>0.76551724165335</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="T19" s="2"/>
+    </row>
+    <row r="20" spans="1:20">
       <c r="A20">
         <v>18</v>
       </c>
@@ -8907,7 +9024,7 @@
         <v>0.74042145616707</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20">
       <c r="A21">
         <v>19</v>
       </c>
@@ -8924,7 +9041,7 @@
         <v>0.75150862096369997</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:20">
       <c r="A22">
         <v>20</v>
       </c>
@@ -8941,7 +9058,7 @@
         <v>0.73575191593718003</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:20">
       <c r="A23">
         <v>21</v>
       </c>
@@ -8958,7 +9075,7 @@
         <v>0.75340038332446002</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:20">
       <c r="A24">
         <v>22</v>
       </c>
@@ -8975,7 +9092,7 @@
         <v>0.72411398503972002</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:20">
       <c r="A25">
         <v>23</v>
       </c>
@@ -8992,7 +9109,7 @@
         <v>0.77140804679913999</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:20">
       <c r="A26">
         <v>24</v>
       </c>
@@ -9009,7 +9126,7 @@
         <v>0.76326628389030005</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20">
       <c r="A27">
         <v>25</v>
       </c>
@@ -9026,7 +9143,7 @@
         <v>0.74738984751975002</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20">
       <c r="A28">
         <v>26</v>
       </c>
@@ -9043,7 +9160,7 @@
         <v>0.76398467469488995</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20">
       <c r="A29">
         <v>27</v>
       </c>
@@ -9060,7 +9177,7 @@
         <v>0.76130268217503005</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20">
       <c r="A30">
         <v>28</v>
       </c>
@@ -9077,7 +9194,7 @@
         <v>0.76537356362945996</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20">
       <c r="A31">
         <v>29</v>
       </c>
@@ -9094,7 +9211,7 @@
         <v>0.76664272053488003</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20">
       <c r="A32">
         <v>30</v>
       </c>
@@ -9111,7 +9228,7 @@
         <v>0.74760536421304002</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5">
       <c r="A33">
         <v>31</v>
       </c>
@@ -9128,7 +9245,7 @@
         <v>0.75433429150746001</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5">
       <c r="A34">
         <v>32</v>
       </c>
@@ -9145,7 +9262,7 @@
         <v>0.75704023070718995</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5">
       <c r="A35">
         <v>33</v>
       </c>
@@ -9162,7 +9279,7 @@
         <v>0.76700191593718003</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5">
       <c r="A36">
         <v>34</v>
       </c>
@@ -9179,7 +9296,7 @@
         <v>0.77306034510163002</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5">
       <c r="A37">
         <v>35</v>
       </c>
@@ -9196,7 +9313,7 @@
         <v>0.76125478950040004</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5">
       <c r="A38">
         <v>36</v>
       </c>
@@ -9213,7 +9330,7 @@
         <v>0.76084770142347002</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5">
       <c r="A39">
         <v>37</v>
       </c>
@@ -9230,7 +9347,7 @@
         <v>0.7710009580371</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5">
       <c r="A40">
         <v>38</v>
       </c>
@@ -9247,7 +9364,7 @@
         <v>0.77787356404051999</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5">
       <c r="A41">
         <v>39</v>
       </c>
@@ -9264,7 +9381,7 @@
         <v>0.74190613045090004</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5">
       <c r="A42">
         <v>40</v>
       </c>
@@ -9281,7 +9398,7 @@
         <v>0.77756226131285999</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5">
       <c r="A43">
         <v>41</v>
       </c>
@@ -9298,7 +9415,7 @@
         <v>0.76992337183020998</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5">
       <c r="A44">
         <v>42</v>
       </c>
@@ -9315,7 +9432,7 @@
         <v>0.76525383160032001</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5">
       <c r="A45">
         <v>43</v>
       </c>
@@ -9332,7 +9449,7 @@
         <v>0.75043103475679995</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5">
       <c r="A46">
         <v>44</v>
       </c>
@@ -9349,7 +9466,7 @@
         <v>0.76357758661796005</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5">
       <c r="A47">
         <v>45</v>
       </c>
@@ -9366,7 +9483,7 @@
         <v>0.72681992355434</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5">
       <c r="A48">
         <v>46</v>
       </c>
@@ -9383,7 +9500,7 @@
         <v>0.77787356404051999</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5">
       <c r="A49">
         <v>47</v>
       </c>
@@ -9400,7 +9517,7 @@
         <v>0.77095306536246999</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5">
       <c r="A50">
         <v>48</v>
       </c>
@@ -9417,7 +9534,7 @@
         <v>0.75816570958871998</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5">
       <c r="A51">
         <v>49</v>
       </c>
@@ -9434,7 +9551,7 @@
         <v>0.76314655254626995</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5">
       <c r="A52">
         <v>50</v>
       </c>
@@ -9451,7 +9568,7 @@
         <v>0.75632183990259005</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5">
       <c r="A53">
         <v>51</v>
       </c>
@@ -9468,7 +9585,7 @@
         <v>0.79875479004849004</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5">
       <c r="A54">
         <v>52</v>
       </c>
@@ -9485,7 +9602,7 @@
         <v>0.77962164769227005</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5">
       <c r="A55">
         <v>53</v>
       </c>
@@ -9502,7 +9619,7 @@
         <v>0.74985632266121005</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5">
       <c r="A56">
         <v>54</v>
       </c>
@@ -9519,7 +9636,7 @@
         <v>0.77418582398316005</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5">
       <c r="A57">
         <v>55</v>
       </c>
@@ -9536,7 +9653,7 @@
         <v>0.79614463619802001</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5">
       <c r="A58">
         <v>56</v>
       </c>
@@ -9553,7 +9670,7 @@
         <v>0.79291187757732995</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5">
       <c r="A59">
         <v>57</v>
       </c>
@@ -9570,7 +9687,7 @@
         <v>0.78900862151178996</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5">
       <c r="A60">
         <v>58</v>
       </c>
@@ -9587,7 +9704,7 @@
         <v>0.77679597783362997</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5">
       <c r="A61">
         <v>59</v>
       </c>
@@ -9604,7 +9721,7 @@
         <v>0.78869731878411997</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5">
       <c r="A62">
         <v>60</v>
       </c>
@@ -9621,7 +9738,7 @@
         <v>0.78223180154273997</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5">
       <c r="A63">
         <v>61</v>
       </c>
@@ -9638,7 +9755,7 @@
         <v>0.78110632266121005</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5">
       <c r="A64">
         <v>62</v>
       </c>
@@ -9655,7 +9772,7 @@
         <v>0.74307950269217005</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5">
       <c r="A65">
         <v>63</v>
       </c>
@@ -9672,7 +9789,7 @@
         <v>0.76853448358075005</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5">
       <c r="A66">
         <v>64</v>
       </c>
@@ -9689,7 +9806,7 @@
         <v>0.77751436863821999</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5">
       <c r="A67">
         <v>65</v>
       </c>
@@ -9706,7 +9823,7 @@
         <v>0.75704023070718995</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5">
       <c r="A68">
         <v>66</v>
       </c>
@@ -9723,7 +9840,7 @@
         <v>0.78685344909800004</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5">
       <c r="A69">
         <v>67</v>
       </c>
@@ -9740,7 +9857,7 @@
         <v>0.78860153274974998</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5">
       <c r="A70">
         <v>68</v>
       </c>
@@ -9757,7 +9874,7 @@
         <v>0.76068007740481003</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5">
       <c r="A71">
         <v>69</v>
       </c>
@@ -9774,7 +9891,7 @@
         <v>0.75488505829340002</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5">
       <c r="A72">
         <v>70</v>
       </c>
@@ -9791,7 +9908,7 @@
         <v>0.79245689682577003</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5">
       <c r="A73">
         <v>71</v>
       </c>
@@ -9808,7 +9925,7 @@
         <v>0.7846982766842</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5">
       <c r="A74">
         <v>72</v>
       </c>
@@ -9825,7 +9942,7 @@
         <v>0.77674808447388</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5">
       <c r="A75">
         <v>73</v>
       </c>
@@ -9842,7 +9959,7 @@
         <v>0.77068965599454997</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:5">
       <c r="A76">
         <v>74</v>
       </c>
@@ -9859,7 +9976,7 @@
         <v>0.74272030728987004</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:5">
       <c r="A77">
         <v>75</v>
       </c>
@@ -9876,7 +9993,7 @@
         <v>0.76278735714396995</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:5">
       <c r="A78">
         <v>76</v>
       </c>
@@ -9893,7 +10010,7 @@
         <v>0.74451628430135997</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:5">
       <c r="A79">
         <v>77</v>
       </c>
@@ -9910,7 +10027,7 @@
         <v>0.76673850656926001</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:5">
       <c r="A80">
         <v>78</v>
       </c>
@@ -9927,7 +10044,7 @@
         <v>0.78393199251986001</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:5">
       <c r="A81">
         <v>79</v>
       </c>
@@ -9944,7 +10061,7 @@
         <v>0.79475574794856996</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:5">
       <c r="A82">
         <v>80</v>
       </c>
@@ -9961,7 +10078,7 @@
         <v>0.77966954105202002</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:5">
       <c r="A83">
         <v>81</v>
       </c>
@@ -9978,7 +10095,7 @@
         <v>0.80095785513691997</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:5">
       <c r="A84">
         <v>82</v>
       </c>
@@ -9995,7 +10112,7 @@
         <v>0.77397030728987004</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:5">
       <c r="A85">
         <v>83</v>
       </c>
@@ -10012,7 +10129,7 @@
         <v>0.78855364007510997</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:5">
       <c r="A86">
         <v>84</v>
       </c>
@@ -10029,7 +10146,7 @@
         <v>0.76489463619802001</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:5">
       <c r="A87">
         <v>85</v>
       </c>
@@ -10046,7 +10163,7 @@
         <v>0.79762931116696001</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:5">
       <c r="A88">
         <v>86</v>
       </c>
@@ -10063,7 +10180,7 @@
         <v>0.76740900401411005</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:5">
       <c r="A89">
         <v>87</v>
       </c>
@@ -10080,7 +10197,7 @@
         <v>0.75857279766565</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:5">
       <c r="A90">
         <v>88</v>
       </c>
@@ -10097,7 +10214,7 @@
         <v>0.78438697395654</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:5">
       <c r="A91">
         <v>89</v>
       </c>
@@ -10114,7 +10231,7 @@
         <v>0.79911398545079004</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:5">
       <c r="A92">
         <v>90</v>
       </c>
@@ -10131,7 +10248,7 @@
         <v>0.78500957872676003</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:5">
       <c r="A93">
         <v>91</v>
       </c>
@@ -10148,7 +10265,7 @@
         <v>0.77500000082213005</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:5">
       <c r="A94">
         <v>92</v>
       </c>
@@ -10165,7 +10282,7 @@
         <v>0.75021551806350995</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:5">
       <c r="A95">
         <v>93</v>
       </c>
@@ -10182,7 +10299,7 @@
         <v>0.74518678243132996</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:5">
       <c r="A96">
         <v>94</v>
       </c>
@@ -10199,7 +10316,7 @@
         <v>0.78397988587959999</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:5">
       <c r="A97">
         <v>95</v>
       </c>
@@ -10216,7 +10333,7 @@
         <v>0.80122126518994996</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:5">
       <c r="A98">
         <v>96</v>
       </c>
@@ -10233,7 +10350,7 @@
         <v>0.80004789294867995</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:5">
       <c r="A99">
         <v>97</v>
       </c>
@@ -10250,7 +10367,7 @@
         <v>0.80615421478775995</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:5">
       <c r="A100">
         <v>98</v>
       </c>
@@ -10267,7 +10384,7 @@
         <v>0.78101053662683995</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:5">
       <c r="A101">
         <v>99</v>
       </c>
@@ -10284,7 +10401,7 @@
         <v>0.79255268217503005</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:5">
       <c r="A102">
         <v>100</v>
       </c>
@@ -10301,7 +10418,7 @@
         <v>0.78208812283372997</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:5">
       <c r="A103">
         <v>101</v>
       </c>
@@ -10318,7 +10435,7 @@
         <v>0.79075670516354002</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:5">
       <c r="A104">
         <v>102</v>
       </c>
@@ -10335,7 +10452,7 @@
         <v>0.75488505829340002</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:5">
       <c r="A105">
         <v>103</v>
       </c>
@@ -10352,7 +10469,7 @@
         <v>0.78675766306362005</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:5">
       <c r="A106">
         <v>104</v>
       </c>
@@ -10369,7 +10486,7 @@
         <v>0.77253352568067002</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:5">
       <c r="A107">
         <v>105</v>
       </c>
@@ -10386,7 +10503,7 @@
         <v>0.79358237570729995</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:5">
       <c r="A108">
         <v>106</v>
       </c>
@@ -10403,7 +10520,7 @@
         <v>0.79655172496005999</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:5">
       <c r="A109">
         <v>107</v>
       </c>
@@ -10420,7 +10537,7 @@
         <v>0.79937739481870995</v>
       </c>
     </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:5">
       <c r="A110">
         <v>108</v>
       </c>
@@ -10437,7 +10554,7 @@
         <v>0.79291187757732995</v>
       </c>
     </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:5">
       <c r="A111">
         <v>109</v>
       </c>
@@ -10454,7 +10571,7 @@
         <v>0.79619252955776998</v>
       </c>
     </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:5">
       <c r="A112">
         <v>110</v>
       </c>
@@ -10471,7 +10588,7 @@
         <v>0.79169061334654001</v>
       </c>
     </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:5">
       <c r="A113">
         <v>111</v>
       </c>
@@ -10488,7 +10605,7 @@
         <v>0.79753352513258002</v>
       </c>
     </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:5">
       <c r="A114">
         <v>112</v>
       </c>
@@ -10505,7 +10622,7 @@
         <v>0.76930076705997996</v>
       </c>
     </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:5">
       <c r="A115">
         <v>113</v>
       </c>
@@ -10522,7 +10639,7 @@
         <v>0.7846982766842</v>
       </c>
     </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:5">
       <c r="A116">
         <v>114</v>
       </c>
@@ -10539,7 +10656,7 @@
         <v>0.80876436863821999</v>
       </c>
     </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:5">
       <c r="A117">
         <v>115</v>
       </c>
@@ -10556,7 +10673,7 @@
         <v>0.81374521091066998</v>
       </c>
     </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:5">
       <c r="A118">
         <v>116</v>
       </c>
@@ -10573,7 +10690,7 @@
         <v>0.78824233734744997</v>
       </c>
     </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:5">
       <c r="A119">
         <v>117</v>
       </c>
@@ -10590,7 +10707,7 @@
         <v>0.80656130286468997</v>
       </c>
     </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:5">
       <c r="A120">
         <v>118</v>
       </c>
@@ -10607,7 +10724,7 @@
         <v>0.80148467455786998</v>
       </c>
     </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:5">
       <c r="A121">
         <v>119</v>
       </c>
@@ -10624,7 +10741,7 @@
         <v>0.79973659022100996</v>
       </c>
     </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:5">
       <c r="A122">
         <v>120</v>
       </c>
@@ -10641,7 +10758,7 @@
         <v>0.78393199251986001</v>
       </c>
     </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:5">
       <c r="A123">
         <v>121</v>
       </c>
@@ -10658,7 +10775,7 @@
         <v>0.80763888907158998</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:5">
       <c r="A124">
         <v>122</v>
       </c>
@@ -10675,7 +10792,7 @@
         <v>0.80368773964630003</v>
       </c>
     </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:5">
       <c r="A125">
         <v>123</v>
       </c>
@@ -10692,7 +10809,7 @@
         <v>0.78613505829340002</v>
       </c>
     </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:5">
       <c r="A126">
         <v>124</v>
       </c>
@@ -10709,7 +10826,7 @@
         <v>0.79121168660021002</v>
       </c>
     </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:5">
       <c r="A127">
         <v>125</v>
       </c>
@@ -10726,7 +10843,7 @@
         <v>0.76843869754637995</v>
       </c>
     </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:5">
       <c r="A128">
         <v>126</v>
       </c>
@@ -10743,7 +10860,7 @@
         <v>0.80620210746238996</v>
       </c>
     </row>
-    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:5">
       <c r="A129">
         <v>127</v>
       </c>
@@ -10760,7 +10877,7 @@
         <v>0.79798850656926001</v>
       </c>
     </row>
-    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:5">
       <c r="A130">
         <v>128</v>
       </c>
@@ -10777,7 +10894,7 @@
         <v>0.79403735714396995</v>
       </c>
     </row>
-    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:5">
       <c r="A131">
         <v>129</v>
       </c>
@@ -10794,7 +10911,7 @@
         <v>0.80871647527848001</v>
       </c>
     </row>
-    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:5">
       <c r="A132">
         <v>130</v>
       </c>
@@ -10811,7 +10928,7 @@
         <v>0.78644636033594995</v>
       </c>
     </row>
-    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:5">
       <c r="A133">
         <v>131</v>
       </c>
@@ -10828,7 +10945,7 @@
         <v>0.82806513432799</v>
       </c>
     </row>
-    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:5">
       <c r="A134">
         <v>132</v>
       </c>
@@ -10845,7 +10962,7 @@
         <v>0.81082375501764004</v>
       </c>
     </row>
-    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:5">
       <c r="A135">
         <v>133</v>
       </c>
@@ -10862,7 +10979,7 @@
         <v>0.77854406148538002</v>
       </c>
     </row>
-    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:5">
       <c r="A136">
         <v>134</v>
       </c>
@@ -10879,7 +10996,7 @@
         <v>0.81056034564972002</v>
       </c>
     </row>
-    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:5">
       <c r="A137">
         <v>135</v>
       </c>
@@ -10896,7 +11013,7 @@
         <v>0.79722222240492002</v>
       </c>
     </row>
-    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:5">
       <c r="A138">
         <v>136</v>
       </c>
@@ -10913,7 +11030,7 @@
         <v>0.78177682010606997</v>
       </c>
     </row>
-    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:5">
       <c r="A139">
         <v>137</v>
       </c>
@@ -10930,7 +11047,7 @@
         <v>0.77274904237396003</v>
       </c>
     </row>
-    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:5">
       <c r="A140">
         <v>138</v>
       </c>
@@ -10947,7 +11064,7 @@
         <v>0.80328065156937001</v>
       </c>
     </row>
-    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:5">
       <c r="A141">
         <v>139</v>
       </c>
@@ -10964,7 +11081,7 @@
         <v>0.81477490444292999</v>
       </c>
     </row>
-    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:5">
       <c r="A142">
         <v>140</v>
       </c>
@@ -10981,7 +11098,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:5">
       <c r="A143">
         <v>141</v>
       </c>
@@ -10998,7 +11115,7 @@
         <v>0.80435823777626003</v>
       </c>
     </row>
-    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:5">
       <c r="A144">
         <v>142</v>
       </c>
@@ -11015,7 +11132,7 @@
         <v>0.80004789294867995</v>
       </c>
     </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:5">
       <c r="A145">
         <v>143</v>
       </c>
@@ -11032,7 +11149,7 @@
         <v>0.80261015343940001</v>
       </c>
     </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:5">
       <c r="A146">
         <v>144</v>
       </c>
@@ -11049,7 +11166,7 @@
         <v>0.79542624539342</v>
       </c>
     </row>
-    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:5">
       <c r="A147">
         <v>145</v>
       </c>
@@ -11066,7 +11183,7 @@
         <v>0.78362069047730998</v>
       </c>
     </row>
-    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:5">
       <c r="A148">
         <v>146</v>
       </c>
@@ -11083,7 +11200,7 @@
         <v>0.81693007685672003</v>
       </c>
     </row>
-    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:5">
       <c r="A149">
         <v>147</v>
       </c>
@@ -11100,7 +11217,7 @@
         <v>0.78393199251986001</v>
       </c>
     </row>
-    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:5">
       <c r="A150">
         <v>148</v>
       </c>
@@ -11117,7 +11234,7 @@
         <v>0.81688218418209002</v>
       </c>
     </row>
-    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:5">
       <c r="A151">
         <v>149</v>
       </c>
@@ -11134,7 +11251,7 @@
         <v>0.80009578562330996</v>
       </c>
     </row>
-    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:5">
       <c r="A152">
         <v>150</v>
       </c>
@@ -11151,7 +11268,7 @@
         <v>0.79727011576466</v>
       </c>
     </row>
-    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:5">
       <c r="A153">
         <v>151</v>
       </c>
@@ -11168,7 +11285,7 @@
         <v>0.80368773964630003</v>
       </c>
     </row>
-    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:5">
       <c r="A154">
         <v>152</v>
       </c>
@@ -11185,7 +11302,7 @@
         <v>0.80040708835097996</v>
       </c>
     </row>
-    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:5">
       <c r="A155">
         <v>153</v>
       </c>
@@ -11202,7 +11319,7 @@
         <v>0.79547413875316997</v>
       </c>
     </row>
-    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:5">
       <c r="A156">
         <v>154</v>
       </c>
@@ -11219,7 +11336,7 @@
         <v>0.80876436863821999</v>
       </c>
     </row>
-    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:5">
       <c r="A157">
         <v>155</v>
       </c>
@@ -11236,7 +11353,7 @@
         <v>0.82528735714396995</v>
       </c>
     </row>
-    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:5">
       <c r="A158">
         <v>156</v>
       </c>
@@ -11253,7 +11370,7 @@
         <v>0.81230842930146996</v>
       </c>
     </row>
-    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:5">
       <c r="A159">
         <v>157</v>
       </c>
@@ -11270,7 +11387,7 @@
         <v>0.81554118792216002</v>
       </c>
     </row>
-    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:5">
       <c r="A160">
         <v>158</v>
       </c>
@@ -11287,7 +11404,7 @@
         <v>0.81774425369570003</v>
       </c>
     </row>
-    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:5">
       <c r="A161">
         <v>159</v>
       </c>
@@ -11304,7 +11421,7 @@
         <v>0.80332854424400002</v>
       </c>
     </row>
-    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:5">
       <c r="A162">
         <v>160</v>
       </c>
@@ -11321,7 +11438,7 @@
         <v>0.81190134122454005</v>
       </c>
     </row>
-    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:5">
       <c r="A163">
         <v>161</v>
       </c>
@@ -11338,7 +11455,7 @@
         <v>0.8155890812819</v>
       </c>
     </row>
-    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:5">
       <c r="A164">
         <v>162</v>
       </c>
@@ -11355,7 +11472,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:5">
       <c r="A165">
         <v>163</v>
       </c>
@@ -11372,7 +11489,7 @@
         <v>0.81087164769227005</v>
       </c>
     </row>
-    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:5">
       <c r="A166">
         <v>164</v>
       </c>
@@ -11389,7 +11506,7 @@
         <v>0.81302682010606997</v>
       </c>
     </row>
-    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:5">
       <c r="A167">
         <v>165</v>
       </c>
@@ -11406,7 +11523,7 @@
         <v>0.80871647527848001</v>
       </c>
     </row>
-    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:5">
       <c r="A168">
         <v>166</v>
       </c>
@@ -11423,7 +11540,7 @@
         <v>0.79121168660021002</v>
       </c>
     </row>
-    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:5">
       <c r="A169">
         <v>167</v>
       </c>
@@ -11440,7 +11557,7 @@
         <v>0.77535919622442995</v>
       </c>
     </row>
-    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:5">
       <c r="A170">
         <v>168</v>
       </c>
@@ -11457,7 +11574,7 @@
         <v>0.81810344909800004</v>
       </c>
     </row>
-    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:5">
       <c r="A171">
         <v>169</v>
       </c>
@@ -11474,7 +11591,7 @@
         <v>0.80727969366928998</v>
       </c>
     </row>
-    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:5">
       <c r="A172">
         <v>170</v>
       </c>
@@ -11491,7 +11608,7 @@
         <v>0.80184386996016999</v>
       </c>
     </row>
-    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:5">
       <c r="A173">
         <v>171</v>
       </c>
@@ -11508,7 +11625,7 @@
         <v>0.79542624539342</v>
       </c>
     </row>
-    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:5">
       <c r="A174">
         <v>172</v>
       </c>
@@ -11525,7 +11642,7 @@
         <v>0.80476532585319005</v>
       </c>
     </row>
-    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:5">
       <c r="A175">
         <v>173</v>
       </c>
@@ -11542,7 +11659,7 @@
         <v>0.79906609277616003</v>
       </c>
     </row>
-    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:5">
       <c r="A176">
         <v>174</v>
       </c>
@@ -11559,7 +11676,7 @@
         <v>0.8018917626348</v>
       </c>
     </row>
-    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:5">
       <c r="A177">
         <v>175</v>
       </c>
@@ -11576,7 +11693,7 @@
         <v>0.79911398545079004</v>
       </c>
     </row>
-    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:5">
       <c r="A178">
         <v>176</v>
       </c>
@@ -11593,7 +11710,7 @@
         <v>0.81621168605213001</v>
       </c>
     </row>
-    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:5">
       <c r="A179">
         <v>177</v>
       </c>
@@ -11610,7 +11727,7 @@
         <v>0.82030651418641998</v>
       </c>
     </row>
-    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:5">
       <c r="A180">
         <v>178</v>
       </c>
@@ -11627,7 +11744,7 @@
         <v>0.81455938774963998</v>
       </c>
     </row>
-    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:5">
       <c r="A181">
         <v>179</v>
       </c>
@@ -11644,7 +11761,7 @@
         <v>0.81482279711756</v>
       </c>
     </row>
-    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:5">
       <c r="A182">
         <v>180</v>
       </c>
@@ -11661,7 +11778,7 @@
         <v>0.80445402381064002</v>
       </c>
     </row>
-    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:5">
       <c r="A183">
         <v>181</v>
       </c>
@@ -11678,7 +11795,7 @@
         <v>0.81815134177263005</v>
       </c>
     </row>
-    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:5">
       <c r="A184">
         <v>182</v>
       </c>
@@ -11695,7 +11812,7 @@
         <v>0.79121168660021002</v>
       </c>
     </row>
-    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:5">
       <c r="A185">
         <v>183</v>
       </c>
@@ -11712,7 +11829,7 @@
         <v>0.79578544079572</v>
       </c>
     </row>
-    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:5">
       <c r="A186">
         <v>184</v>
       </c>
@@ -11729,7 +11846,7 @@
         <v>0.79583333415546997</v>
       </c>
     </row>
-    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:5">
       <c r="A187">
         <v>185</v>
       </c>
@@ -11746,7 +11863,7 @@
         <v>0.77684387050825998</v>
       </c>
     </row>
-    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:5">
       <c r="A188">
         <v>186</v>
       </c>
@@ -11763,7 +11880,7 @@
         <v>0.79475574794856996</v>
       </c>
     </row>
-    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:5">
       <c r="A189">
         <v>187</v>
       </c>
@@ -11780,7 +11897,7 @@
         <v>0.79897030674178005</v>
       </c>
     </row>
-    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:5">
       <c r="A190">
         <v>188</v>
       </c>
@@ -11797,7 +11914,7 @@
         <v>0.80009578562330996</v>
       </c>
     </row>
-    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:5">
       <c r="A191">
         <v>189</v>
       </c>
@@ -11814,7 +11931,7 @@
         <v>0.78465038332446002</v>
       </c>
     </row>
-    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:5">
       <c r="A192">
         <v>190</v>
       </c>
@@ -11831,7 +11948,7 @@
         <v>0.81271551806350995</v>
       </c>
     </row>
-    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:5">
       <c r="A193">
         <v>191</v>
       </c>
@@ -11848,7 +11965,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:5">
       <c r="A194">
         <v>192</v>
       </c>
@@ -11865,7 +11982,7 @@
         <v>0.80126915786457997</v>
       </c>
     </row>
-    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:5">
       <c r="A195">
         <v>193</v>
       </c>
@@ -11882,7 +11999,7 @@
         <v>0.80373563300604001</v>
       </c>
     </row>
-    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:5">
       <c r="A196">
         <v>194</v>
       </c>
@@ -11899,7 +12016,7 @@
         <v>0.81446360171526</v>
       </c>
     </row>
-    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:5">
       <c r="A197">
         <v>195</v>
       </c>
@@ -11916,7 +12033,7 @@
         <v>0.82488026838192996</v>
       </c>
     </row>
-    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:5">
       <c r="A198">
         <v>196</v>
       </c>
@@ -11933,7 +12050,7 @@
         <v>0.81343390886810996</v>
       </c>
     </row>
-    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:5">
       <c r="A199">
         <v>197</v>
       </c>
@@ -11950,7 +12067,7 @@
         <v>0.81046455961534003</v>
       </c>
     </row>
-    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:5">
       <c r="A200">
         <v>198</v>
       </c>
@@ -11967,7 +12084,7 @@
         <v>0.77746647527848001</v>
       </c>
     </row>
-    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:5">
       <c r="A201">
         <v>199</v>
       </c>
@@ -11984,7 +12101,7 @@
         <v>0.77746647527848001</v>
       </c>
     </row>
-    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:5">
       <c r="A202">
         <v>200</v>
       </c>
@@ -12001,7 +12118,7 @@
         <v>0.79798850656926001</v>
       </c>
     </row>
-    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:5">
       <c r="A203">
         <v>201</v>
       </c>
@@ -12018,7 +12135,7 @@
         <v>0.80435823777626003</v>
       </c>
     </row>
-    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:5">
       <c r="A204">
         <v>202</v>
       </c>
@@ -12035,7 +12152,7 @@
         <v>0.80953065211746</v>
       </c>
     </row>
-    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:5">
       <c r="A205">
         <v>203</v>
       </c>
@@ -12052,7 +12169,7 @@
         <v>0.81882183990259005</v>
       </c>
     </row>
-    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:5">
       <c r="A206">
         <v>204</v>
       </c>
@@ -12069,7 +12186,7 @@
         <v>0.81235632266121005</v>
       </c>
     </row>
-    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:5">
       <c r="A207">
         <v>205</v>
       </c>
@@ -12086,7 +12203,7 @@
         <v>0.80696839162672995</v>
       </c>
     </row>
-    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:5">
       <c r="A208">
         <v>206</v>
       </c>
@@ -12103,7 +12220,7 @@
         <v>0.82492816174167005</v>
       </c>
     </row>
-    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:5">
       <c r="A209">
         <v>207</v>
       </c>
@@ -12120,7 +12237,7 @@
         <v>0.83278256723249999</v>
       </c>
     </row>
-    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:5">
       <c r="A210">
         <v>208</v>
       </c>
@@ -12137,7 +12254,7 @@
         <v>0.81702586289110002</v>
       </c>
     </row>
-    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:5">
       <c r="A211">
         <v>209</v>
       </c>
@@ -12154,7 +12271,7 @@
         <v>0.8159482766842</v>
       </c>
     </row>
-    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:5">
       <c r="A212">
         <v>210</v>
       </c>
@@ -12171,7 +12288,7 @@
         <v>0.81482279711756</v>
       </c>
     </row>
-    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:5">
       <c r="A213">
         <v>211</v>
       </c>
@@ -12188,7 +12305,7 @@
         <v>0.82420977093708003</v>
       </c>
     </row>
-    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:5">
       <c r="A214">
         <v>212</v>
       </c>
@@ -12205,7 +12322,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:5">
       <c r="A215">
         <v>213</v>
       </c>
@@ -12222,7 +12339,7 @@
         <v>0.79753352513258002</v>
       </c>
     </row>
-    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:5">
       <c r="A216">
         <v>214</v>
       </c>
@@ -12239,7 +12356,7 @@
         <v>0.79327107297962995</v>
       </c>
     </row>
-    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:5">
       <c r="A217">
         <v>215</v>
       </c>
@@ -12256,7 +12373,7 @@
         <v>0.81841475114054996</v>
       </c>
     </row>
-    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:5">
       <c r="A218">
         <v>216</v>
       </c>
@@ -12273,7 +12390,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:5">
       <c r="A219">
         <v>217</v>
       </c>
@@ -12290,7 +12407,7 @@
         <v>0.81297892743143996</v>
       </c>
     </row>
-    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:5">
       <c r="A220">
         <v>218</v>
       </c>
@@ -12307,7 +12424,7 @@
         <v>0.82667624539342</v>
       </c>
     </row>
-    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:5">
       <c r="A221">
         <v>219</v>
       </c>
@@ -12324,7 +12441,7 @@
         <v>0.82586206923955996</v>
       </c>
     </row>
-    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:5">
       <c r="A222">
         <v>220</v>
       </c>
@@ -12341,7 +12458,7 @@
         <v>0.82088122628200999</v>
       </c>
     </row>
-    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:5">
       <c r="A223">
         <v>221</v>
       </c>
@@ -12358,7 +12475,7 @@
         <v>0.82236590056584002</v>
       </c>
     </row>
-    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:5">
       <c r="A224">
         <v>222</v>
       </c>
@@ -12375,7 +12492,7 @@
         <v>0.80301724220144</v>
       </c>
     </row>
-    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:5">
       <c r="A225">
         <v>223</v>
       </c>
@@ -12392,7 +12509,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:5">
       <c r="A226">
         <v>224</v>
       </c>
@@ -12409,7 +12526,7 @@
         <v>0.8155890812819</v>
       </c>
     </row>
-    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:5">
       <c r="A227">
         <v>225</v>
       </c>
@@ -12426,7 +12543,7 @@
         <v>0.81451149507500997</v>
       </c>
     </row>
-    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:5">
       <c r="A228">
         <v>226</v>
       </c>
@@ -12443,7 +12560,7 @@
         <v>0.80917145671516</v>
       </c>
     </row>
-    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:5">
       <c r="A229">
         <v>227</v>
       </c>
@@ -12460,7 +12577,7 @@
         <v>0.80593869809447005</v>
       </c>
     </row>
-    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:5">
       <c r="A230">
         <v>228</v>
       </c>
@@ -12477,7 +12594,7 @@
         <v>0.82030651418641998</v>
       </c>
     </row>
-    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:5">
       <c r="A231">
         <v>229</v>
       </c>
@@ -12494,7 +12611,7 @@
         <v>0.81815134177263005</v>
       </c>
     </row>
-    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:5">
       <c r="A232">
         <v>230</v>
       </c>
@@ -12511,7 +12628,7 @@
         <v>0.80198754866917998</v>
       </c>
     </row>
-    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:5">
       <c r="A233">
         <v>231</v>
       </c>
@@ -12528,7 +12645,7 @@
         <v>0.81240421533585006</v>
       </c>
     </row>
-    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:5">
       <c r="A234">
         <v>232</v>
       </c>
@@ -12545,7 +12662,7 @@
         <v>0.80732758702902996</v>
       </c>
     </row>
-    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:5">
       <c r="A235">
         <v>233</v>
       </c>
@@ -12562,7 +12679,7 @@
         <v>0.79188218473018002</v>
       </c>
     </row>
-    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:5">
       <c r="A236">
         <v>234</v>
       </c>
@@ -12579,7 +12696,7 @@
         <v>0.80445402381064002</v>
       </c>
     </row>
-    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:5">
       <c r="A237">
         <v>235</v>
       </c>
@@ -12596,7 +12713,7 @@
         <v>0.80517241461524003</v>
       </c>
     </row>
-    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:5">
       <c r="A238">
         <v>236</v>
       </c>
@@ -12613,7 +12730,7 @@
         <v>0.80557950269217005</v>
       </c>
     </row>
-    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:5">
       <c r="A239">
         <v>237</v>
       </c>
@@ -12630,7 +12747,7 @@
         <v>0.80696839162672995</v>
       </c>
     </row>
-    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:5">
       <c r="A240">
         <v>238</v>
       </c>
@@ -12647,7 +12764,7 @@
         <v>0.81810344909800004</v>
       </c>
     </row>
-    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:5">
       <c r="A241">
         <v>239</v>
       </c>
@@ -12664,7 +12781,7 @@
         <v>0.78007662912895004</v>
       </c>
     </row>
-    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:5">
       <c r="A242">
         <v>240</v>
       </c>
@@ -12681,7 +12798,7 @@
         <v>0.81702586289110002</v>
       </c>
     </row>
-    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:5">
       <c r="A243">
         <v>241</v>
       </c>
@@ -12698,7 +12815,7 @@
         <v>0.82852011576466</v>
       </c>
     </row>
-    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:5">
       <c r="A244">
         <v>242</v>
       </c>
@@ -12715,7 +12832,7 @@
         <v>0.81697796953136004</v>
       </c>
     </row>
-    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:5">
       <c r="A245">
         <v>243</v>
       </c>
@@ -12732,7 +12849,7 @@
         <v>0.81343390886810996</v>
       </c>
     </row>
-    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:5">
       <c r="A246">
         <v>244</v>
       </c>
@@ -12749,7 +12866,7 @@
         <v>0.82097701231638998</v>
       </c>
     </row>
-    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:5">
       <c r="A247">
         <v>245</v>
       </c>
@@ -12766,7 +12883,7 @@
         <v>0.81846264450029005</v>
       </c>
     </row>
-    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:5">
       <c r="A248">
         <v>246</v>
       </c>
@@ -12783,7 +12900,7 @@
         <v>0.82349138013248002</v>
       </c>
     </row>
-    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:5">
       <c r="A249">
         <v>247</v>
       </c>
@@ -12800,7 +12917,7 @@
         <v>0.82600574794856996</v>
       </c>
     </row>
-    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:5">
       <c r="A250">
         <v>248</v>
       </c>
@@ -12817,7 +12934,7 @@
         <v>0.79363026838192996</v>
       </c>
     </row>
-    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:5">
       <c r="A251">
         <v>249</v>
       </c>
@@ -12834,7 +12951,7 @@
         <v>0.79588122683009999</v>
       </c>
     </row>
-    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:5">
       <c r="A252">
         <v>250</v>
       </c>
@@ -12851,7 +12968,7 @@
         <v>0.80553161001754003</v>
       </c>
     </row>
-    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:5">
       <c r="A253">
         <v>251</v>
       </c>
@@ -12868,7 +12985,7 @@
         <v>0.81918103530488995</v>
       </c>
     </row>
-    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:5">
       <c r="A254">
         <v>252</v>
       </c>
@@ -12885,7 +13002,7 @@
         <v>0.80409482840834001</v>
       </c>
     </row>
-    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:5">
       <c r="A255">
         <v>253</v>
       </c>
@@ -12902,7 +13019,7 @@
         <v>0.80198754866917998</v>
       </c>
     </row>
-    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="256" spans="1:5">
       <c r="A256">
         <v>254</v>
       </c>
@@ -12919,7 +13036,7 @@
         <v>0.81127873645432003</v>
       </c>
     </row>
-    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="257" spans="1:5">
       <c r="A257">
         <v>255</v>
       </c>
@@ -12936,7 +13053,7 @@
         <v>0.81388888961966999</v>
       </c>
     </row>
-    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="258" spans="1:5">
       <c r="A258">
         <v>256</v>
       </c>
@@ -12953,7 +13070,7 @@
         <v>0.82174329579562</v>
       </c>
     </row>
-    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="259" spans="1:5">
       <c r="A259">
         <v>257</v>
       </c>
@@ -12970,7 +13087,7 @@
         <v>0.81163793185662003</v>
       </c>
     </row>
-    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="260" spans="1:5">
       <c r="A260">
         <v>258</v>
       </c>
@@ -12987,7 +13104,7 @@
         <v>0.80414272108297002</v>
       </c>
     </row>
-    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="261" spans="1:5">
       <c r="A261">
         <v>259</v>
       </c>
@@ -13004,7 +13121,7 @@
         <v>0.80229885139684998</v>
       </c>
     </row>
-    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="262" spans="1:5">
       <c r="A262">
         <v>260</v>
       </c>
@@ -13021,7 +13138,7 @@
         <v>0.81096743372665003</v>
       </c>
     </row>
-    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="263" spans="1:5">
       <c r="A263">
         <v>261</v>
       </c>
@@ -13038,7 +13155,7 @@
         <v>0.81949233734744997</v>
       </c>
     </row>
-    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="264" spans="1:5">
       <c r="A264">
         <v>262</v>
       </c>
@@ -13055,7 +13172,7 @@
         <v>0.80737547970365997</v>
       </c>
     </row>
-    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="265" spans="1:5">
       <c r="A265">
         <v>263</v>
       </c>
@@ -13072,7 +13189,7 @@
         <v>0.82143199306795001</v>
       </c>
     </row>
-    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="266" spans="1:5">
       <c r="A266">
         <v>264</v>
       </c>
@@ -13089,7 +13206,7 @@
         <v>0.80814176318288999</v>
       </c>
     </row>
-    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="267" spans="1:5">
       <c r="A267">
         <v>265</v>
       </c>
@@ -13106,7 +13223,7 @@
         <v>0.81168582453125004</v>
       </c>
     </row>
-    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:5">
       <c r="A268">
         <v>266</v>
       </c>
@@ -13123,7 +13240,7 @@
         <v>0.82564655254626995</v>
       </c>
     </row>
-    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="269" spans="1:5">
       <c r="A269">
         <v>267</v>
       </c>
@@ -13140,7 +13257,7 @@
         <v>0.828208813037</v>
       </c>
     </row>
-    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="270" spans="1:5">
       <c r="A270">
         <v>268</v>
       </c>
@@ -13157,7 +13274,7 @@
         <v>0.83287835326687998</v>
       </c>
     </row>
-    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="271" spans="1:5">
       <c r="A271">
         <v>269</v>
       </c>
@@ -13174,7 +13291,7 @@
         <v>0.80993774019439002</v>
       </c>
     </row>
-    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="272" spans="1:5">
       <c r="A272">
         <v>270</v>
       </c>
@@ -13191,7 +13308,7 @@
         <v>0.81671456016343003</v>
       </c>
     </row>
-    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="273" spans="1:5">
       <c r="A273">
         <v>271</v>
       </c>
@@ -13208,7 +13325,7 @@
         <v>0.81348180154273997</v>
       </c>
     </row>
-    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="274" spans="1:5">
       <c r="A274">
         <v>272</v>
       </c>
@@ -13225,7 +13342,7 @@
         <v>0.80270593947377999</v>
       </c>
     </row>
-    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="275" spans="1:5">
       <c r="A275">
         <v>273</v>
       </c>
@@ -13242,7 +13359,7 @@
         <v>0.81168582453125004</v>
       </c>
     </row>
-    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="276" spans="1:5">
       <c r="A276">
         <v>274</v>
       </c>
@@ -13259,7 +13376,7 @@
         <v>0.80162835326687998</v>
       </c>
     </row>
-    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="277" spans="1:5">
       <c r="A277">
         <v>275</v>
       </c>
@@ -13276,7 +13393,7 @@
         <v>0.81630747208650001</v>
       </c>
     </row>
-    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="278" spans="1:5">
       <c r="A278">
         <v>276</v>
       </c>
@@ -13293,7 +13410,7 @@
         <v>0.81522988587959999</v>
       </c>
     </row>
-    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="279" spans="1:5">
       <c r="A279">
         <v>277</v>
       </c>
@@ -13310,7 +13427,7 @@
         <v>0.82097701231638998</v>
       </c>
     </row>
-    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="280" spans="1:5">
       <c r="A280">
         <v>278</v>
       </c>
@@ -13327,7 +13444,7 @@
         <v>0.80948275944282</v>
       </c>
     </row>
-    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:5">
       <c r="A281">
         <v>279</v>
       </c>
@@ -13344,7 +13461,7 @@
         <v>0.8155890812819</v>
       </c>
     </row>
-    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="282" spans="1:5">
       <c r="A282">
         <v>280</v>
       </c>
@@ -13361,7 +13478,7 @@
         <v>0.80378352568067002</v>
       </c>
     </row>
-    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="283" spans="1:5">
       <c r="A283">
         <v>281</v>
       </c>
@@ -13378,7 +13495,7 @@
         <v>0.82061781691408997</v>
       </c>
     </row>
-    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="284" spans="1:5">
       <c r="A284">
         <v>282</v>
       </c>
@@ -13395,7 +13512,7 @@
         <v>0.81994731878411997</v>
       </c>
     </row>
-    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="285" spans="1:5">
       <c r="A285">
         <v>283</v>
       </c>
@@ -13412,7 +13529,7 @@
         <v>0.80957854479209002</v>
       </c>
     </row>
-    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="286" spans="1:5">
       <c r="A286">
         <v>284</v>
       </c>
@@ -13429,7 +13546,7 @@
         <v>0.80953065211746</v>
       </c>
     </row>
-    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="287" spans="1:5">
       <c r="A287">
         <v>285</v>
       </c>
@@ -13446,7 +13563,7 @@
         <v>0.81851053717493005</v>
       </c>
     </row>
-    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="288" spans="1:5">
       <c r="A288">
         <v>286</v>
       </c>
@@ -13463,7 +13580,7 @@
         <v>0.81199712725891005</v>
       </c>
     </row>
-    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="289" spans="1:5">
       <c r="A289">
         <v>287</v>
       </c>
@@ -13480,7 +13597,7 @@
         <v>0.82222222254194</v>
       </c>
     </row>
-    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="290" spans="1:5">
       <c r="A290">
         <v>288</v>
       </c>
@@ -13497,7 +13614,7 @@
         <v>0.82205459852328</v>
       </c>
     </row>
-    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="291" spans="1:5">
       <c r="A291">
         <v>289</v>
       </c>
@@ -13514,7 +13631,7 @@
         <v>0.82097701231638998</v>
       </c>
     </row>
-    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="292" spans="1:5">
       <c r="A292">
         <v>290</v>
       </c>
@@ -13531,7 +13648,7 @@
         <v>0.82600574794856996</v>
       </c>
     </row>
-    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="293" spans="1:5">
       <c r="A293">
         <v>291</v>
       </c>
@@ -13548,7 +13665,7 @@
         <v>0.83965517323592997</v>
       </c>
     </row>
-    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:5">
       <c r="A294">
         <v>292</v>
       </c>
@@ -13565,7 +13682,7 @@
         <v>0.82385057553478003</v>
       </c>
     </row>
-    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="295" spans="1:5">
       <c r="A295">
         <v>293</v>
       </c>
@@ -13582,7 +13699,7 @@
         <v>0.82744252955776998</v>
       </c>
     </row>
-    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="296" spans="1:5">
       <c r="A296">
         <v>294</v>
       </c>
@@ -13599,7 +13716,7 @@
         <v>0.83144157165768995</v>
       </c>
     </row>
-    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="297" spans="1:5">
       <c r="A297">
         <v>295</v>
       </c>
@@ -13616,7 +13733,7 @@
         <v>0.81851053717493005</v>
       </c>
     </row>
-    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="298" spans="1:5">
       <c r="A298">
         <v>296</v>
       </c>
@@ -13633,7 +13750,7 @@
         <v>0.82353927280711003</v>
       </c>
     </row>
-    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="299" spans="1:5">
       <c r="A299">
         <v>297</v>
       </c>
@@ -13650,7 +13767,7 @@
         <v>0.83144157165768995</v>
       </c>
     </row>
-    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="300" spans="1:5">
       <c r="A300">
         <v>298</v>
       </c>
@@ -13667,7 +13784,7 @@
         <v>0.81235632266121005</v>
       </c>
     </row>
-    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="301" spans="1:5">
       <c r="A301">
         <v>299</v>
       </c>
@@ -13684,7 +13801,7 @@
         <v>0.82852011576466</v>
       </c>
     </row>
-    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="302" spans="1:5">
       <c r="A302">
         <v>300</v>
       </c>
@@ -13701,7 +13818,7 @@
         <v>0.81199712725891005</v>
       </c>
     </row>
-    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="303" spans="1:5">
       <c r="A303">
         <v>301</v>
       </c>
@@ -13718,7 +13835,7 @@
         <v>0.83175287438534995</v>
       </c>
     </row>
-    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="304" spans="1:5">
       <c r="A304">
         <v>302</v>
       </c>
@@ -13735,7 +13852,7 @@
         <v>0.83318965599454997</v>
       </c>
     </row>
-    <row r="305" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="305" spans="1:5">
       <c r="A305">
         <v>303</v>
       </c>
@@ -13752,7 +13869,7 @@
         <v>0.83072318085309005</v>
       </c>
     </row>
-    <row r="306" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="306" spans="1:5">
       <c r="A306">
         <v>304</v>
       </c>
@@ -13769,7 +13886,7 @@
         <v>0.82641283602549998</v>
       </c>
     </row>
-    <row r="307" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:5">
       <c r="A307">
         <v>305</v>
       </c>
@@ -13786,7 +13903,7 @@
         <v>0.81989942610948996</v>
       </c>
     </row>
-    <row r="308" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="308" spans="1:5">
       <c r="A308">
         <v>306</v>
       </c>
@@ -13803,7 +13920,7 @@
         <v>0.82528735714396995</v>
       </c>
     </row>
-    <row r="309" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="309" spans="1:5">
       <c r="A309">
         <v>307</v>
       </c>
@@ -13820,7 +13937,7 @@
         <v>0.83031609277616003</v>
       </c>
     </row>
-    <row r="310" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="310" spans="1:5">
       <c r="A310">
         <v>308</v>
       </c>
@@ -13837,7 +13954,7 @@
         <v>0.82856800843929002</v>
       </c>
     </row>
-    <row r="311" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="311" spans="1:5">
       <c r="A311">
         <v>309</v>
       </c>
@@ -13854,7 +13971,7 @@
         <v>0.81144636047298002</v>
       </c>
     </row>
-    <row r="312" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="312" spans="1:5">
       <c r="A312">
         <v>310</v>
       </c>
@@ -13871,7 +13988,7 @@
         <v>0.83709291206008996</v>
       </c>
     </row>
-    <row r="313" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="313" spans="1:5">
       <c r="A313">
         <v>311</v>
       </c>
@@ -13888,7 +14005,7 @@
         <v>0.83426724220144</v>
       </c>
     </row>
-    <row r="314" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="314" spans="1:5">
       <c r="A314">
         <v>312</v>
       </c>
@@ -13905,7 +14022,7 @@
         <v>0.81810344909800004</v>
       </c>
     </row>
-    <row r="315" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="315" spans="1:5">
       <c r="A315">
         <v>313</v>
       </c>
@@ -13922,7 +14039,7 @@
         <v>0.82272509596814003</v>
       </c>
     </row>
-    <row r="316" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="316" spans="1:5">
       <c r="A316">
         <v>314</v>
       </c>
@@ -13939,7 +14056,7 @@
         <v>0.82437739495573004</v>
       </c>
     </row>
-    <row r="317" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="317" spans="1:5">
       <c r="A317">
         <v>315</v>
       </c>
@@ -13956,7 +14073,7 @@
         <v>0.83920019179924998</v>
       </c>
     </row>
-    <row r="318" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="318" spans="1:5">
       <c r="A318">
         <v>316</v>
       </c>
@@ -13973,7 +14090,7 @@
         <v>0.82313218473018002</v>
       </c>
     </row>
-    <row r="319" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="319" spans="1:5">
       <c r="A319">
         <v>317</v>
       </c>
@@ -13990,7 +14107,7 @@
         <v>0.83426724220144</v>
       </c>
     </row>
-    <row r="320" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:5">
       <c r="A320">
         <v>318</v>
       </c>
@@ -14007,7 +14124,7 @@
         <v>0.82030651418641998</v>
       </c>
     </row>
-    <row r="321" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="321" spans="1:5">
       <c r="A321">
         <v>319</v>
       </c>
@@ -14024,7 +14141,7 @@
         <v>0.82456896633937005</v>
       </c>
     </row>
-    <row r="322" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="322" spans="1:5">
       <c r="A322">
         <v>320</v>
       </c>
@@ -14041,7 +14158,7 @@
         <v>0.82456896633937005</v>
       </c>
     </row>
-    <row r="323" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="323" spans="1:5">
       <c r="A323">
         <v>321</v>
       </c>
@@ -14058,7 +14175,7 @@
         <v>0.81707375556573003</v>
       </c>
     </row>
-    <row r="324" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="324" spans="1:5">
       <c r="A324">
         <v>322</v>
       </c>
@@ -14075,7 +14192,7 @@
         <v>0.82636494335086996</v>
       </c>
     </row>
-    <row r="325" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="325" spans="1:5">
       <c r="A325">
         <v>323</v>
       </c>
@@ -14092,7 +14209,7 @@
         <v>0.83031609277616003</v>
       </c>
     </row>
-    <row r="326" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="326" spans="1:5">
       <c r="A326">
         <v>324</v>
       </c>
@@ -14109,7 +14226,7 @@
         <v>0.83642241461524003</v>
       </c>
     </row>
-    <row r="327" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="327" spans="1:5">
       <c r="A327">
         <v>325</v>
       </c>
@@ -14126,7 +14243,7 @@
         <v>0.82061781691408997</v>
       </c>
     </row>
-    <row r="328" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="328" spans="1:5">
       <c r="A328">
         <v>326</v>
       </c>
@@ -14143,7 +14260,7 @@
         <v>0.81415229967270997</v>
       </c>
     </row>
-    <row r="329" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="329" spans="1:5">
       <c r="A329">
         <v>327</v>
       </c>
@@ -14160,7 +14277,7 @@
         <v>0.82564655254626995</v>
       </c>
     </row>
-    <row r="330" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="330" spans="1:5">
       <c r="A330">
         <v>328</v>
       </c>
@@ -14177,7 +14294,7 @@
         <v>0.83283046059224997</v>
       </c>
     </row>
-    <row r="331" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="331" spans="1:5">
       <c r="A331">
         <v>329</v>
       </c>
@@ -14194,7 +14311,7 @@
         <v>0.84216954105202002</v>
       </c>
     </row>
-    <row r="332" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="332" spans="1:5">
       <c r="A332">
         <v>330</v>
       </c>
@@ -14211,7 +14328,7 @@
         <v>0.83606321921294002</v>
       </c>
     </row>
-    <row r="333" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:5">
       <c r="A333">
         <v>331</v>
       </c>
@@ -14228,7 +14345,7 @@
         <v>0.80907567068078001</v>
       </c>
     </row>
-    <row r="334" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="334" spans="1:5">
       <c r="A334">
         <v>332</v>
       </c>
@@ -14245,7 +14362,7 @@
         <v>0.81522988587959999</v>
       </c>
     </row>
-    <row r="335" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="335" spans="1:5">
       <c r="A335">
         <v>333</v>
       </c>
@@ -14262,7 +14379,7 @@
         <v>0.81738505829340002</v>
       </c>
     </row>
-    <row r="336" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="336" spans="1:5">
       <c r="A336">
         <v>334</v>
       </c>
@@ -14279,7 +14396,7 @@
         <v>0.82667624539342</v>
       </c>
     </row>
-    <row r="337" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="337" spans="1:5">
       <c r="A337">
         <v>335</v>
       </c>
@@ -14296,7 +14413,7 @@
         <v>0.82241379392558001</v>
       </c>
     </row>
-    <row r="338" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="338" spans="1:5">
       <c r="A338">
         <v>336</v>
       </c>
@@ -14313,7 +14430,7 @@
         <v>0.81989942610948996</v>
       </c>
     </row>
-    <row r="339" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="339" spans="1:5">
       <c r="A339">
         <v>337</v>
       </c>
@@ -14330,7 +14447,7 @@
         <v>0.81446360171526</v>
       </c>
     </row>
-    <row r="340" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="340" spans="1:5">
       <c r="A340">
         <v>338</v>
       </c>
@@ -14347,7 +14464,7 @@
         <v>0.80948275944282</v>
       </c>
     </row>
-    <row r="341" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="341" spans="1:5">
       <c r="A341">
         <v>339</v>
       </c>
@@ -14364,7 +14481,7 @@
         <v>0.82523946378422997</v>
       </c>
     </row>
-    <row r="342" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="342" spans="1:5">
       <c r="A342">
         <v>340</v>
       </c>
@@ -14381,7 +14498,7 @@
         <v>0.81877394654284996</v>
       </c>
     </row>
-    <row r="343" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="343" spans="1:5">
       <c r="A343">
         <v>341</v>
       </c>
@@ -14398,7 +14515,7 @@
         <v>0.82770593892569</v>
       </c>
     </row>
-    <row r="344" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="344" spans="1:5">
       <c r="A344">
         <v>342</v>
       </c>
@@ -14415,7 +14532,7 @@
         <v>0.82344348677273005</v>
       </c>
     </row>
-    <row r="345" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="345" spans="1:5">
       <c r="A345">
         <v>343</v>
       </c>
@@ -14432,7 +14549,7 @@
         <v>0.83026819941640995</v>
       </c>
     </row>
-    <row r="346" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:5">
       <c r="A346">
         <v>344</v>
       </c>
@@ -14449,7 +14566,7 @@
         <v>0.83098659022100996</v>
       </c>
     </row>
-    <row r="347" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="347" spans="1:5">
       <c r="A347">
         <v>345</v>
       </c>
@@ -14466,7 +14583,7 @@
         <v>0.80440613045090004</v>
       </c>
     </row>
-    <row r="348" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="348" spans="1:5">
       <c r="A348">
         <v>346</v>
       </c>
@@ -14483,7 +14600,7 @@
         <v>0.82954980861182004</v>
       </c>
     </row>
-    <row r="349" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="349" spans="1:5">
       <c r="A349">
         <v>347</v>
       </c>
@@ -14500,7 +14617,7 @@
         <v>0.83263888920860996</v>
       </c>
     </row>
-    <row r="350" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="350" spans="1:5">
       <c r="A350">
         <v>348</v>
       </c>
@@ -14517,7 +14634,7 @@
         <v>0.82954980861182004</v>
       </c>
     </row>
-    <row r="351" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="351" spans="1:5">
       <c r="A351">
         <v>349</v>
       </c>
@@ -14534,7 +14651,7 @@
         <v>0.81159003849686995</v>
       </c>
     </row>
-    <row r="352" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="352" spans="1:5">
       <c r="A352">
         <v>350</v>
       </c>
@@ -14551,7 +14668,7 @@
         <v>0.80040708835097996</v>
       </c>
     </row>
-    <row r="353" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="353" spans="1:5">
       <c r="A353">
         <v>351</v>
       </c>
@@ -14568,7 +14685,7 @@
         <v>0.81805555573824995</v>
       </c>
     </row>
-    <row r="354" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="354" spans="1:5">
       <c r="A354">
         <v>352</v>
       </c>
@@ -14585,7 +14702,7 @@
         <v>0.82025862151178996</v>
       </c>
     </row>
-    <row r="355" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="355" spans="1:5">
       <c r="A355">
         <v>353</v>
       </c>
@@ -14602,7 +14719,7 @@
         <v>0.82092911895664</v>
       </c>
     </row>
-    <row r="356" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="356" spans="1:5">
       <c r="A356">
         <v>354</v>
       </c>
@@ -14619,7 +14736,7 @@
         <v>0.82775383160032001</v>
       </c>
     </row>
-    <row r="357" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="357" spans="1:5">
       <c r="A357">
         <v>355</v>
       </c>
@@ -14636,7 +14753,7 @@
         <v>0.82447318030500005</v>
       </c>
     </row>
-    <row r="358" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="358" spans="1:5">
       <c r="A358">
         <v>356</v>
       </c>
@@ -14653,7 +14770,7 @@
         <v>0.82344348677273005</v>
       </c>
     </row>
-    <row r="359" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:5">
       <c r="A359">
         <v>357</v>
       </c>
@@ -14670,7 +14787,7 @@
         <v>0.81702586289110002</v>
       </c>
     </row>
-    <row r="360" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="360" spans="1:5">
       <c r="A360">
         <v>358</v>
       </c>
@@ -14687,7 +14804,7 @@
         <v>0.81056034564972002</v>
       </c>
     </row>
-    <row r="361" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="361" spans="1:5">
       <c r="A361">
         <v>359</v>
       </c>
@@ -14704,7 +14821,7 @@
         <v>0.82744252955776998</v>
       </c>
     </row>
-    <row r="362" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="362" spans="1:5">
       <c r="A362">
         <v>360</v>
       </c>
@@ -14721,7 +14838,7 @@
         <v>0.81415229967270997</v>
       </c>
     </row>
-    <row r="363" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="363" spans="1:5">
       <c r="A363">
         <v>361</v>
       </c>
@@ -14738,7 +14855,7 @@
         <v>0.83283046059224997</v>
       </c>
     </row>
-    <row r="364" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="364" spans="1:5">
       <c r="A364">
         <v>362</v>
       </c>
@@ -14755,7 +14872,7 @@
         <v>0.82780172496005999</v>
       </c>
     </row>
-    <row r="365" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="365" spans="1:5">
       <c r="A365">
         <v>363</v>
       </c>
@@ -14772,7 +14889,7 @@
         <v>0.82816092036236</v>
       </c>
     </row>
-    <row r="366" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="366" spans="1:5">
       <c r="A366">
         <v>364</v>
       </c>
@@ -14789,7 +14906,7 @@
         <v>0.82313218473018002</v>
       </c>
     </row>
-    <row r="367" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="367" spans="1:5">
       <c r="A367">
         <v>365</v>
       </c>
@@ -14806,7 +14923,7 @@
         <v>0.82241379392558001</v>
       </c>
     </row>
-    <row r="368" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="368" spans="1:5">
       <c r="A368">
         <v>366</v>
       </c>
@@ -14823,7 +14940,7 @@
         <v>0.81127873645432003</v>
       </c>
     </row>
-    <row r="369" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="369" spans="1:5">
       <c r="A369">
         <v>367</v>
       </c>
@@ -14840,7 +14957,7 @@
         <v>0.82097701231638998</v>
       </c>
     </row>
-    <row r="370" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="370" spans="1:5">
       <c r="A370">
         <v>368</v>
       </c>
@@ -14857,7 +14974,7 @@
         <v>0.79516283602549998</v>
       </c>
     </row>
-    <row r="371" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="371" spans="1:5">
       <c r="A371">
         <v>369</v>
       </c>
@@ -14874,7 +14991,7 @@
         <v>0.81199712725891005</v>
       </c>
     </row>
-    <row r="372" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:5">
       <c r="A372">
         <v>370</v>
       </c>
@@ -14891,7 +15008,7 @@
         <v>0.81522988587959999</v>
       </c>
     </row>
-    <row r="373" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="373" spans="1:5">
       <c r="A373">
         <v>371</v>
       </c>
@@ -14908,7 +15025,7 @@
         <v>0.80876436863821999</v>
       </c>
     </row>
-    <row r="374" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="374" spans="1:5">
       <c r="A374">
         <v>372</v>
       </c>
@@ -14925,7 +15042,7 @@
         <v>0.81774425369570003</v>
       </c>
     </row>
-    <row r="375" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="375" spans="1:5">
       <c r="A375">
         <v>373</v>
       </c>
@@ -14942,7 +15059,7 @@
         <v>0.81168582453125004</v>
       </c>
     </row>
-    <row r="376" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="376" spans="1:5">
       <c r="A376">
         <v>374</v>
       </c>
@@ -14959,7 +15076,7 @@
         <v>0.81487069047730998</v>
       </c>
     </row>
-    <row r="377" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="377" spans="1:5">
       <c r="A377">
         <v>375</v>
       </c>
@@ -14976,7 +15093,7 @@
         <v>0.81810344909800004</v>
       </c>
     </row>
-    <row r="378" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="378" spans="1:5">
       <c r="A378">
         <v>376</v>
       </c>
@@ -14993,7 +15110,7 @@
         <v>0.81882183990259005</v>
       </c>
     </row>
-    <row r="379" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="379" spans="1:5">
       <c r="A379">
         <v>377</v>
       </c>
@@ -15010,7 +15127,7 @@
         <v>0.81779214637033004</v>
       </c>
     </row>
-    <row r="380" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="380" spans="1:5">
       <c r="A380">
         <v>378</v>
       </c>
@@ -15027,7 +15144,7 @@
         <v>0.82954980861182004</v>
       </c>
     </row>
-    <row r="381" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="381" spans="1:5">
       <c r="A381">
         <v>379</v>
       </c>
@@ -15044,7 +15161,7 @@
         <v>0.81477490444292999</v>
       </c>
     </row>
-    <row r="382" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="382" spans="1:5">
       <c r="A382">
         <v>380</v>
       </c>
@@ -15061,7 +15178,7 @@
         <v>0.81374521091066998</v>
       </c>
     </row>
-    <row r="383" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="383" spans="1:5">
       <c r="A383">
         <v>381</v>
       </c>
@@ -15078,7 +15195,7 @@
         <v>0.82703544079572</v>
       </c>
     </row>
-    <row r="384" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="384" spans="1:5">
       <c r="A384">
         <v>382</v>
       </c>
@@ -15095,7 +15212,7 @@
         <v>0.80763888907158998</v>
       </c>
     </row>
-    <row r="385" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:5">
       <c r="A385">
         <v>383</v>
       </c>
@@ -15112,7 +15229,7 @@
         <v>0.82780172496005999</v>
       </c>
     </row>
-    <row r="386" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="386" spans="1:5">
       <c r="A386">
         <v>384</v>
       </c>
@@ -15129,7 +15246,7 @@
         <v>0.82456896633937005</v>
       </c>
     </row>
-    <row r="387" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="387" spans="1:5">
       <c r="A387">
         <v>385</v>
       </c>
@@ -15146,7 +15263,7 @@
         <v>0.83318965599454997</v>
       </c>
     </row>
-    <row r="388" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="388" spans="1:5">
       <c r="A388">
         <v>386</v>
       </c>
@@ -15163,7 +15280,7 @@
         <v>0.82492816174167005</v>
       </c>
     </row>
-    <row r="389" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="389" spans="1:5">
       <c r="A389">
         <v>387</v>
       </c>
@@ -15180,7 +15297,7 @@
         <v>0.82174329579562</v>
       </c>
     </row>
-    <row r="390" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="390" spans="1:5">
       <c r="A390">
         <v>388</v>
       </c>
@@ -15197,7 +15314,7 @@
         <v>0.81779214637033004</v>
       </c>
     </row>
-    <row r="391" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="391" spans="1:5">
       <c r="A391">
         <v>389</v>
       </c>
@@ -15214,7 +15331,7 @@
         <v>0.81563697395654</v>
       </c>
     </row>
-    <row r="392" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="392" spans="1:5">
       <c r="A392">
         <v>390</v>
       </c>
@@ -15231,7 +15348,7 @@
         <v>0.80840517323592997</v>
       </c>
     </row>
-    <row r="393" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="393" spans="1:5">
       <c r="A393">
         <v>391</v>
       </c>
@@ -15248,7 +15365,7 @@
         <v>0.81994731878411997</v>
       </c>
     </row>
-    <row r="394" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="394" spans="1:5">
       <c r="A394">
         <v>392</v>
       </c>
@@ -15265,7 +15382,7 @@
         <v>0.82138410039331999</v>
       </c>
     </row>
-    <row r="395" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="395" spans="1:5">
       <c r="A395">
         <v>393</v>
       </c>
@@ -15282,7 +15399,7 @@
         <v>0.81671456016343003</v>
       </c>
     </row>
-    <row r="396" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="396" spans="1:5">
       <c r="A396">
         <v>394</v>
       </c>
@@ -15299,7 +15416,7 @@
         <v>0.82492816174167005</v>
       </c>
     </row>
-    <row r="397" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="397" spans="1:5">
       <c r="A397">
         <v>395</v>
       </c>
@@ -15316,7 +15433,7 @@
         <v>0.81676245283806004</v>
       </c>
     </row>
-    <row r="398" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:5">
       <c r="A398">
         <v>396</v>
       </c>
@@ -15333,7 +15450,7 @@
         <v>0.80917145671516</v>
       </c>
     </row>
-    <row r="399" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="399" spans="1:5">
       <c r="A399">
         <v>397</v>
       </c>
@@ -15350,7 +15467,7 @@
         <v>0.82605364062319997</v>
       </c>
     </row>
-    <row r="400" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="400" spans="1:5">
       <c r="A400">
         <v>398</v>
       </c>
@@ -15367,7 +15484,7 @@
         <v>0.83242337183020998</v>
       </c>
     </row>
-    <row r="401" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="401" spans="1:5">
       <c r="A401">
         <v>399</v>
       </c>
@@ -15384,7 +15501,7 @@
         <v>0.82349138013248002</v>
       </c>
     </row>
-    <row r="402" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="402" spans="1:5">
       <c r="A402">
         <v>400</v>
       </c>
@@ -15401,7 +15518,7 @@
         <v>0.83472222295301002</v>
       </c>
     </row>
-    <row r="403" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="403" spans="1:5">
       <c r="A403">
         <v>401</v>
       </c>
@@ -15418,7 +15535,7 @@
         <v>0.82806513432799</v>
       </c>
     </row>
-    <row r="404" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="404" spans="1:5">
       <c r="A404">
         <v>402</v>
       </c>
@@ -15435,7 +15552,7 @@
         <v>0.82919061320952003</v>
       </c>
     </row>
-    <row r="405" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="405" spans="1:5">
       <c r="A405">
         <v>403</v>
       </c>
@@ -15452,7 +15569,7 @@
         <v>0.80696839162672995</v>
       </c>
     </row>
-    <row r="406" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="406" spans="1:5">
       <c r="A406">
         <v>404</v>
       </c>
@@ -15469,7 +15586,7 @@
         <v>0.828208813037</v>
       </c>
     </row>
-    <row r="407" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="407" spans="1:5">
       <c r="A407">
         <v>405</v>
       </c>
@@ -15486,7 +15603,7 @@
         <v>0.83144157165768995</v>
       </c>
     </row>
-    <row r="408" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="408" spans="1:5">
       <c r="A408">
         <v>406</v>
       </c>
@@ -15503,7 +15620,7 @@
         <v>0.82856800843929002</v>
       </c>
     </row>
-    <row r="409" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="409" spans="1:5">
       <c r="A409">
         <v>407</v>
       </c>
@@ -15520,7 +15637,7 @@
         <v>0.83000479004849004</v>
       </c>
     </row>
-    <row r="410" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="410" spans="1:5">
       <c r="A410">
         <v>408</v>
       </c>
@@ -15537,7 +15654,7 @@
         <v>0.82502394709093996</v>
       </c>
     </row>
-    <row r="411" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:5">
       <c r="A411">
         <v>409</v>
       </c>
@@ -15554,7 +15671,7 @@
         <v>0.82713122683009999</v>
       </c>
     </row>
-    <row r="412" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="412" spans="1:5">
       <c r="A412">
         <v>410</v>
       </c>
@@ -15571,7 +15688,7 @@
         <v>0.81420019234733998</v>
       </c>
     </row>
-    <row r="413" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="413" spans="1:5">
       <c r="A413">
         <v>411</v>
       </c>
@@ -15588,7 +15705,7 @@
         <v>0.81599616935883001</v>
       </c>
     </row>
-    <row r="414" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="414" spans="1:5">
       <c r="A414">
         <v>412</v>
       </c>
@@ -15605,7 +15722,7 @@
         <v>0.82909482786025002</v>
       </c>
     </row>
-    <row r="415" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="415" spans="1:5">
       <c r="A415">
         <v>413</v>
       </c>
@@ -15622,7 +15739,7 @@
         <v>0.82928639924389003</v>
       </c>
     </row>
-    <row r="416" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="416" spans="1:5">
       <c r="A416">
         <v>414</v>
       </c>
@@ -15639,7 +15756,7 @@
         <v>0.82749042223239999</v>
       </c>
     </row>
-    <row r="417" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="417" spans="1:5">
       <c r="A417">
         <v>415</v>
       </c>
@@ -15656,7 +15773,7 @@
         <v>0.81635536476113002</v>
       </c>
     </row>
-    <row r="418" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="418" spans="1:5">
       <c r="A418">
         <v>416</v>
       </c>
@@ -15673,7 +15790,7 @@
         <v>0.82286877467715003</v>
       </c>
     </row>
-    <row r="419" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="419" spans="1:5">
       <c r="A419">
         <v>417</v>
       </c>
@@ -15690,7 +15807,7 @@
         <v>0.83750000082213005</v>
       </c>
     </row>
-    <row r="420" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="420" spans="1:5">
       <c r="A420">
         <v>418</v>
       </c>
@@ -15707,7 +15824,7 @@
         <v>0.83503352568067002</v>
       </c>
     </row>
-    <row r="421" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="421" spans="1:5">
       <c r="A421">
         <v>419</v>
       </c>
@@ -15724,7 +15841,7 @@
         <v>0.82461685901401005</v>
       </c>
     </row>
-    <row r="422" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="422" spans="1:5">
       <c r="A422">
         <v>420</v>
       </c>
@@ -15741,7 +15858,7 @@
         <v>0.82389846820941004</v>
       </c>
     </row>
-    <row r="423" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="423" spans="1:5">
       <c r="A423">
         <v>421</v>
       </c>
@@ -15758,7 +15875,7 @@
         <v>0.81168582453125004</v>
       </c>
     </row>
-    <row r="424" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:5">
       <c r="A424">
         <v>422</v>
       </c>
@@ -15775,7 +15892,7 @@
         <v>0.83323754866917998</v>
       </c>
     </row>
-    <row r="425" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="425" spans="1:5">
       <c r="A425">
         <v>423</v>
       </c>
@@ -15792,7 +15909,7 @@
         <v>0.83139367898305006</v>
       </c>
     </row>
-    <row r="426" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="426" spans="1:5">
       <c r="A426">
         <v>424</v>
       </c>
@@ -15809,7 +15926,7 @@
         <v>0.81810344909800004</v>
       </c>
     </row>
-    <row r="427" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="427" spans="1:5">
       <c r="A427">
         <v>425</v>
       </c>
@@ -15826,7 +15943,7 @@
         <v>0.81343390886810996</v>
       </c>
     </row>
-    <row r="428" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="428" spans="1:5">
       <c r="A428">
         <v>426</v>
       </c>
@@ -15843,7 +15960,7 @@
         <v>0.82461685901401005</v>
       </c>
     </row>
-    <row r="429" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="429" spans="1:5">
       <c r="A429">
         <v>427</v>
       </c>
@@ -15860,7 +15977,7 @@
         <v>0.82744252955776998</v>
       </c>
     </row>
-    <row r="430" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="430" spans="1:5">
       <c r="A430">
         <v>428</v>
       </c>
@@ -15877,7 +15994,7 @@
         <v>0.82923850656926001</v>
       </c>
     </row>
-    <row r="431" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="431" spans="1:5">
       <c r="A431">
         <v>429</v>
       </c>
@@ -15894,7 +16011,7 @@
         <v>0.82964559464619003</v>
       </c>
     </row>
-    <row r="432" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="432" spans="1:5">
       <c r="A432">
         <v>430</v>
       </c>
@@ -15911,7 +16028,7 @@
         <v>0.82923850656926001</v>
       </c>
     </row>
-    <row r="433" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="433" spans="1:5">
       <c r="A433">
         <v>431</v>
       </c>
@@ -15928,7 +16045,7 @@
         <v>0.82349138013248002</v>
       </c>
     </row>
-    <row r="434" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="434" spans="1:5">
       <c r="A434">
         <v>432</v>
       </c>
@@ -15945,7 +16062,7 @@
         <v>0.82456896633937005</v>
       </c>
     </row>
-    <row r="435" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="435" spans="1:5">
       <c r="A435">
         <v>433</v>
       </c>
@@ -15962,7 +16079,7 @@
         <v>0.81815134177263005</v>
       </c>
     </row>
-    <row r="436" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="436" spans="1:5">
       <c r="A436">
         <v>434</v>
       </c>
@@ -15979,7 +16096,7 @@
         <v>0.83287835326687998</v>
       </c>
     </row>
-    <row r="437" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:5">
       <c r="A437">
         <v>435</v>
       </c>
@@ -15996,7 +16113,7 @@
         <v>0.83031609277616003</v>
       </c>
     </row>
-    <row r="438" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="438" spans="1:5">
       <c r="A438">
         <v>436</v>
       </c>
@@ -16013,7 +16130,7 @@
         <v>0.83251915786457997</v>
       </c>
     </row>
-    <row r="439" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="439" spans="1:5">
       <c r="A439">
         <v>437</v>
       </c>
@@ -16030,7 +16147,7 @@
         <v>0.82461685901401005</v>
       </c>
     </row>
-    <row r="440" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="440" spans="1:5">
       <c r="A440">
         <v>438</v>
       </c>
@@ -16047,7 +16164,7 @@
         <v>0.83108237625539005</v>
       </c>
     </row>
-    <row r="441" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="441" spans="1:5">
       <c r="A441">
         <v>439</v>
       </c>
@@ -16064,7 +16181,7 @@
         <v>0.82569444522089996</v>
       </c>
     </row>
-    <row r="442" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="442" spans="1:5">
       <c r="A442">
         <v>440</v>
       </c>
@@ -16081,7 +16198,7 @@
         <v>0.83036398545079004</v>
       </c>
     </row>
-    <row r="443" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="443" spans="1:5">
       <c r="A443">
         <v>441</v>
       </c>
@@ -16098,7 +16215,7 @@
         <v>0.82502394709093996</v>
       </c>
     </row>
-    <row r="444" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="444" spans="1:5">
       <c r="A444">
         <v>442</v>
       </c>
@@ -16115,7 +16232,7 @@
         <v>0.83539272108297002</v>
       </c>
     </row>
-    <row r="445" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="445" spans="1:5">
       <c r="A445">
         <v>443</v>
       </c>
@@ -16132,7 +16249,7 @@
         <v>0.83139367898305006</v>
       </c>
     </row>
-    <row r="446" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="446" spans="1:5">
       <c r="A446">
         <v>444</v>
       </c>
@@ -16149,7 +16266,7 @@
         <v>0.80598659076909995</v>
       </c>
     </row>
-    <row r="447" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="447" spans="1:5">
       <c r="A447">
         <v>445</v>
       </c>
@@ -16166,7 +16283,7 @@
         <v>0.81922892797951996</v>
       </c>
     </row>
-    <row r="448" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="448" spans="1:5">
       <c r="A448">
         <v>446</v>
       </c>
@@ -16183,7 +16300,7 @@
         <v>0.828208813037</v>
       </c>
     </row>
-    <row r="449" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="449" spans="1:5">
       <c r="A449">
         <v>447</v>
       </c>
@@ -16200,7 +16317,7 @@
         <v>0.82246168660021002</v>
       </c>
     </row>
-    <row r="450" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:5">
       <c r="A450">
         <v>448</v>
       </c>
@@ -16217,7 +16334,7 @@
         <v>0.82286877467715003</v>
       </c>
     </row>
-    <row r="451" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="451" spans="1:5">
       <c r="A451">
         <v>449</v>
       </c>
@@ -16234,7 +16351,7 @@
         <v>0.80670498157369996</v>
       </c>
     </row>
-    <row r="452" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="452" spans="1:5">
       <c r="A452">
         <v>450</v>
       </c>
@@ -16251,7 +16368,7 @@
         <v>0.78726053717493005</v>
       </c>
     </row>
-    <row r="453" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="453" spans="1:5">
       <c r="A453">
         <v>451</v>
       </c>
@@ -16268,7 +16385,7 @@
         <v>0.81307471346580995</v>
       </c>
     </row>
-    <row r="454" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="454" spans="1:5">
       <c r="A454">
         <v>452</v>
       </c>
@@ -16285,7 +16402,7 @@
         <v>0.81985153274974998</v>
       </c>
     </row>
-    <row r="455" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="455" spans="1:5">
       <c r="A455">
         <v>453</v>
       </c>
@@ -16302,7 +16419,7 @@
         <v>0.81738505829340002</v>
       </c>
     </row>
-    <row r="456" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="456" spans="1:5">
       <c r="A456">
         <v>454</v>
       </c>
@@ -16319,7 +16436,7 @@
         <v>0.81922892797951996</v>
       </c>
     </row>
-    <row r="457" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="457" spans="1:5">
       <c r="A457">
         <v>455</v>
       </c>
@@ -16336,7 +16453,7 @@
         <v>0.81841475114054996</v>
       </c>
     </row>
-    <row r="458" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="458" spans="1:5">
       <c r="A458">
         <v>456</v>
       </c>
@@ -16353,7 +16470,7 @@
         <v>0.81410440631295999</v>
       </c>
     </row>
-    <row r="459" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="459" spans="1:5">
       <c r="A459">
         <v>457</v>
       </c>
@@ -16370,7 +16487,7 @@
         <v>0.80984195484512</v>
       </c>
     </row>
-    <row r="460" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="460" spans="1:5">
       <c r="A460">
         <v>458</v>
       </c>
@@ -16387,7 +16504,7 @@
         <v>0.82564655254626995</v>
       </c>
     </row>
-    <row r="461" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="461" spans="1:5">
       <c r="A461">
         <v>459</v>
       </c>
@@ -16404,7 +16521,7 @@
         <v>0.82066570958871998</v>
       </c>
     </row>
-    <row r="462" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="462" spans="1:5">
       <c r="A462">
         <v>460</v>
       </c>
@@ -16421,7 +16538,7 @@
         <v>0.81338601550836998</v>
       </c>
     </row>
-    <row r="463" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:5">
       <c r="A463">
         <v>461</v>
       </c>
@@ -16438,7 +16555,7 @@
         <v>0.8155890812819</v>
       </c>
     </row>
-    <row r="464" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="464" spans="1:5">
       <c r="A464">
         <v>462</v>
       </c>
@@ -16455,7 +16572,7 @@
         <v>0.82600574794856996</v>
       </c>
     </row>
-    <row r="465" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="465" spans="1:5">
       <c r="A465">
         <v>463</v>
       </c>
@@ -16472,7 +16589,7 @@
         <v>0.82236590056584002</v>
       </c>
     </row>
-    <row r="466" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="466" spans="1:5">
       <c r="A466">
         <v>464</v>
       </c>
@@ -16489,7 +16606,7 @@
         <v>0.83036398545079004</v>
       </c>
     </row>
-    <row r="467" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="467" spans="1:5">
       <c r="A467">
         <v>465</v>
       </c>
@@ -16506,7 +16623,7 @@
         <v>0.82739463619802001</v>
       </c>
     </row>
-    <row r="468" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="468" spans="1:5">
       <c r="A468">
         <v>466</v>
       </c>
@@ -16523,7 +16640,7 @@
         <v>0.82919061320952003</v>
       </c>
     </row>
-    <row r="469" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="469" spans="1:5">
       <c r="A469">
         <v>467</v>
       </c>
@@ -16540,7 +16657,7 @@
         <v>0.83026819941640995</v>
       </c>
     </row>
-    <row r="470" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="470" spans="1:5">
       <c r="A470">
         <v>468</v>
       </c>
@@ -16557,7 +16674,7 @@
         <v>0.83170498102560997</v>
       </c>
     </row>
-    <row r="471" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="471" spans="1:5">
       <c r="A471">
         <v>469</v>
       </c>
@@ -16574,7 +16691,7 @@
         <v>0.82631704999112998</v>
       </c>
     </row>
-    <row r="472" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="472" spans="1:5">
       <c r="A472">
         <v>470</v>
       </c>
@@ -16591,7 +16708,7 @@
         <v>0.83709291206008996</v>
       </c>
     </row>
-    <row r="473" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="473" spans="1:5">
       <c r="A473">
         <v>471</v>
       </c>
@@ -16608,7 +16725,7 @@
         <v>0.83376436809013998</v>
       </c>
     </row>
-    <row r="474" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="474" spans="1:5">
       <c r="A474">
         <v>472</v>
       </c>
@@ -16625,7 +16742,7 @@
         <v>0.83556034510163002</v>
       </c>
     </row>
-    <row r="475" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="475" spans="1:5">
       <c r="A475">
         <v>473</v>
       </c>
@@ -16642,7 +16759,7 @@
         <v>0.83453065156937001</v>
       </c>
     </row>
-    <row r="476" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:5">
       <c r="A476">
         <v>474</v>
       </c>
@@ -16659,7 +16776,7 @@
         <v>0.83165708835097996</v>
       </c>
     </row>
-    <row r="477" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="477" spans="1:5">
       <c r="A477">
         <v>475</v>
       </c>
@@ -16676,7 +16793,7 @@
         <v>0.82452107297962995</v>
       </c>
     </row>
-    <row r="478" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="478" spans="1:5">
       <c r="A478">
         <v>476</v>
       </c>
@@ -16693,7 +16810,7 @@
         <v>0.82339559409810004</v>
       </c>
     </row>
-    <row r="479" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="479" spans="1:5">
       <c r="A479">
         <v>477</v>
       </c>
@@ -16710,7 +16827,7 @@
         <v>0.83534482840834001</v>
       </c>
     </row>
-    <row r="480" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="480" spans="1:5">
       <c r="A480">
         <v>478</v>
       </c>
@@ -16727,7 +16844,7 @@
         <v>0.82698754812108999</v>
       </c>
     </row>
-    <row r="481" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="481" spans="1:5">
       <c r="A481">
         <v>479</v>
       </c>
@@ -16744,7 +16861,7 @@
         <v>0.82442528763037004</v>
       </c>
     </row>
-    <row r="482" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="482" spans="1:5">
       <c r="A482">
         <v>480</v>
       </c>
@@ -16761,7 +16878,7 @@
         <v>0.83057950214408005</v>
       </c>
     </row>
-    <row r="483" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="483" spans="1:5">
       <c r="A483">
         <v>481</v>
       </c>
@@ -16778,7 +16895,7 @@
         <v>0.82887931116696001</v>
       </c>
     </row>
-    <row r="484" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="484" spans="1:5">
       <c r="A484">
         <v>482</v>
       </c>
@@ -16795,7 +16912,7 @@
         <v>0.83498563300604001</v>
       </c>
     </row>
-    <row r="485" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="485" spans="1:5">
       <c r="A485">
         <v>483</v>
       </c>
@@ -16812,7 +16929,7 @@
         <v>0.82420977093708003</v>
       </c>
     </row>
-    <row r="486" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="486" spans="1:5">
       <c r="A486">
         <v>484</v>
       </c>
@@ -16829,7 +16946,7 @@
         <v>0.83103448358075005</v>
       </c>
     </row>
-    <row r="487" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="487" spans="1:5">
       <c r="A487">
         <v>485</v>
       </c>
@@ -16846,7 +16963,7 @@
         <v>0.81805555573824995</v>
       </c>
     </row>
-    <row r="488" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="488" spans="1:5">
       <c r="A488">
         <v>486</v>
       </c>
@@ -16863,7 +16980,7 @@
         <v>0.82344348677273005</v>
       </c>
     </row>
-    <row r="489" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:5">
       <c r="A489">
         <v>487</v>
       </c>
@@ -16880,7 +16997,7 @@
         <v>0.82646072870012999</v>
       </c>
     </row>
-    <row r="490" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="490" spans="1:5">
       <c r="A490">
         <v>488</v>
       </c>
@@ -16897,7 +17014,7 @@
         <v>0.83287835326687998</v>
       </c>
     </row>
-    <row r="491" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="491" spans="1:5">
       <c r="A491">
         <v>489</v>
       </c>
@@ -16914,7 +17031,7 @@
         <v>0.82739463619802001</v>
       </c>
     </row>
-    <row r="492" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="492" spans="1:5">
       <c r="A492">
         <v>490</v>
       </c>
@@ -16931,7 +17048,7 @@
         <v>0.82523946378422997</v>
       </c>
     </row>
-    <row r="493" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="493" spans="1:5">
       <c r="A493">
         <v>491</v>
       </c>
@@ -16948,7 +17065,7 @@
         <v>0.83000479004849004</v>
       </c>
     </row>
-    <row r="494" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="494" spans="1:5">
       <c r="A494">
         <v>492</v>
       </c>
@@ -16965,7 +17082,7 @@
         <v>0.82708333415546997</v>
       </c>
     </row>
-    <row r="495" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="495" spans="1:5">
       <c r="A495">
         <v>493</v>
       </c>
@@ -16982,7 +17099,7 @@
         <v>0.82928639924389003</v>
       </c>
     </row>
-    <row r="496" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="496" spans="1:5">
       <c r="A496">
         <v>494</v>
       </c>
@@ -16999,7 +17116,7 @@
         <v>0.82569444522089996</v>
       </c>
     </row>
-    <row r="497" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="497" spans="1:5">
       <c r="A497">
         <v>495</v>
       </c>
@@ -17016,7 +17133,7 @@
         <v>0.83170498102560997</v>
       </c>
     </row>
-    <row r="498" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="498" spans="1:5">
       <c r="A498">
         <v>496</v>
       </c>
@@ -17033,7 +17150,7 @@
         <v>0.83129789294867995</v>
       </c>
     </row>
-    <row r="499" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="499" spans="1:5">
       <c r="A499">
         <v>497</v>
       </c>
@@ -17050,7 +17167,7 @@
         <v>0.83318965599454997</v>
       </c>
     </row>
-    <row r="500" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="500" spans="1:5">
       <c r="A500">
         <v>498</v>
       </c>
@@ -17067,7 +17184,7 @@
         <v>0.81635536476113002</v>
       </c>
     </row>
-    <row r="501" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="501" spans="1:5">
       <c r="A501">
         <v>499</v>
       </c>
@@ -17087,6 +17204,7 @@
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>